<commit_message>
fix(AIM-4684): financial model + doc consistency (review findings)
- Weekly Ramp sheet: AppExchange rev-share now respects ent_checkout param
  (base case 0% direct sales) — App D €31.5k, SUMME €117.1k, consistent
  with Overview/Portfolio/CSV
- business-plan: App D contribution €31.5k (was €26k)
- risk-register R12: gap €31.5k (was €26k)
- scoring matrix: pre-fill scores recomputed per documented formula
  (85/86/78/66, 0-100 scale), scale note + Watchlist rationale for App D
- KPI dashboard: install target 1.000/wk (derived from model ramp at 3%
  conversion), formula footnote
</commit_message>
<xml_diff>
--- a/docs/gtm/marketplace-arbitrage/financial-model.xlsx
+++ b/docs/gtm/marketplace-arbitrage/financial-model.xlsx
@@ -1340,7 +1340,7 @@
         <v>3500</v>
       </c>
       <c r="H5" t="n">
-        <v>26759.26</v>
+        <v>31481.48</v>
       </c>
     </row>
     <row r="6">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr"/>
       <c r="H7" s="2" t="n">
-        <v>112410.14</v>
+        <v>117132.36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>